<commit_message>
Regression test case completed +ve flow of code
</commit_message>
<xml_diff>
--- a/com.dot.app/src/test/resources/TestData.xlsx
+++ b/com.dot.app/src/test/resources/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\Feb\com.dot.app\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A0304F-27D7-4692-B20C-6BF4B1559C15}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{956A3810-8547-4484-A9AD-E6A58E84A894}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15360" windowHeight="1080" tabRatio="869" activeTab="8" xr2:uid="{FEC993B8-5DA9-4590-A44D-BF2ACF9ACFC9}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="108">
   <si>
     <t>TestCaseName</t>
   </si>
@@ -358,9 +358,6 @@
     <t>defectPriority</t>
   </si>
   <si>
-    <t>medium</t>
-  </si>
-  <si>
     <t>deleteDefect</t>
   </si>
   <si>
@@ -368,6 +365,9 @@
   </si>
   <si>
     <t>Open</t>
+  </si>
+  <si>
+    <t>Medium</t>
   </si>
 </sst>
 </file>
@@ -2023,7 +2023,7 @@
         <v>75</v>
       </c>
       <c r="J3" s="5">
-        <v>3262025</v>
+        <v>4022025</v>
       </c>
       <c r="K3" t="s">
         <v>82</v>
@@ -2080,7 +2080,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDFDCB89-E8A6-448C-BC83-AD5BDE959D4B}">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
@@ -2093,9 +2093,10 @@
     <col min="8" max="10" width="9.90625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="19.6328125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -2135,8 +2136,11 @@
       <c r="M1" s="7" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="N1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="14" t="s">
         <v>84</v>
       </c>
@@ -2154,19 +2158,19 @@
         <v>101</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="J2">
         <v>1</v>
       </c>
       <c r="K2">
-        <v>3262025</v>
+        <v>4022025</v>
       </c>
       <c r="L2" t="s">
         <v>59</v>
@@ -2174,8 +2178,11 @@
       <c r="M2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="N2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="16" t="s">
         <v>85</v>
       </c>
@@ -2207,7 +2214,7 @@
         <v>102</v>
       </c>
       <c r="K3">
-        <v>3272025</v>
+        <v>4022025</v>
       </c>
       <c r="L3" t="s">
         <v>75</v>
@@ -2215,10 +2222,13 @@
       <c r="M3" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="N3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="20" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B4" s="21" t="s">
         <v>5</v>
@@ -2229,7 +2239,9 @@
       <c r="D4" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="E4" s="13"/>
+      <c r="E4" t="s">
+        <v>75</v>
+      </c>
       <c r="F4" s="8" t="s">
         <v>75</v>
       </c>
@@ -2253,6 +2265,53 @@
       </c>
       <c r="M4" s="8" t="s">
         <v>75</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="N5" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -2263,6 +2322,8 @@
     <hyperlink ref="C3" r:id="rId4" xr:uid="{B9758A73-3C1B-4D66-BD63-4F678EBEC6C6}"/>
     <hyperlink ref="B4" r:id="rId5" xr:uid="{7EC821D7-6690-4FA4-AA84-D4E595BD56AF}"/>
     <hyperlink ref="C4" r:id="rId6" xr:uid="{59ABF189-C279-4D80-A47D-451BF16A05C8}"/>
+    <hyperlink ref="B5" r:id="rId7" xr:uid="{6D13F3A2-A89C-453A-B0B4-35A84AFB0735}"/>
+    <hyperlink ref="C5" r:id="rId8" xr:uid="{21692565-C8EF-4BA4-AB9E-C255898AADFE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>